<commit_message>
Added Features : Local First Geosensing, live order history, money-map, other fixes
</commit_message>
<xml_diff>
--- a/backend/reports/users_report.xlsx
+++ b/backend/reports/users_report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="76">
   <si>
     <t>#</t>
   </si>
@@ -57,169 +57,115 @@
     <t>+91-9988776655</t>
   </si>
   <si>
-    <t>—</t>
+    <t>Brigade Road, Bengaluru</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>₹450.00</t>
+    <t>₹0.00</t>
   </si>
   <si>
     <t>Active</t>
   </si>
   <si>
-    <t>3/3/2026, 3:50:40 pm</t>
-  </si>
-  <si>
-    <t>Tom Cruise</t>
-  </si>
-  <si>
-    <t>tom@impossible.com</t>
-  </si>
-  <si>
-    <t>010145</t>
-  </si>
-  <si>
-    <t>₹341.00</t>
-  </si>
-  <si>
-    <t>3/3/2026, 5:27:04 pm</t>
-  </si>
-  <si>
-    <t>Test Buyer</t>
-  </si>
-  <si>
-    <t>testbuyer123@example.com</t>
-  </si>
-  <si>
-    <t>1234567890</t>
-  </si>
-  <si>
-    <t>₹185.00</t>
-  </si>
-  <si>
-    <t>3/3/2026, 7:29:22 pm</t>
-  </si>
-  <si>
-    <t>Ravi</t>
-  </si>
-  <si>
-    <t>ravi@mnit.ac.in</t>
-  </si>
-  <si>
-    <t>123456</t>
+    <t>4/3/2026, 10:29:44 pm</t>
+  </si>
+  <si>
+    <t>Sneha Rao</t>
+  </si>
+  <si>
+    <t>sneha@buyer.com</t>
+  </si>
+  <si>
+    <t>+91-9988776666</t>
+  </si>
+  <si>
+    <t>Domlur, Bengaluru</t>
+  </si>
+  <si>
+    <t>Rohan Gupta</t>
+  </si>
+  <si>
+    <t>rohan@buyer.com</t>
+  </si>
+  <si>
+    <t>+91-9988776677</t>
+  </si>
+  <si>
+    <t>India Gate vicinity, New Delhi</t>
+  </si>
+  <si>
+    <t>4/3/2026, 10:29:45 pm</t>
+  </si>
+  <si>
+    <t>Maya Patel</t>
+  </si>
+  <si>
+    <t>maya@buyer.com</t>
+  </si>
+  <si>
+    <t>+91-9988776688</t>
+  </si>
+  <si>
+    <t>Colaba, Mumbai</t>
+  </si>
+  <si>
+    <t>Jaipur User</t>
+  </si>
+  <si>
+    <t>jaipur@buyer.com</t>
+  </si>
+  <si>
+    <t>+91-9000000000</t>
+  </si>
+  <si>
+    <t>C-Scheme, Jaipur, Rajasthan</t>
+  </si>
+  <si>
+    <t>Shop Name</t>
+  </si>
+  <si>
+    <t>Shop Category</t>
+  </si>
+  <si>
+    <t>Shop Address</t>
+  </si>
+  <si>
+    <t>Shop Verified</t>
+  </si>
+  <si>
+    <t>Shop Open</t>
+  </si>
+  <si>
+    <t>Shop Rating</t>
+  </si>
+  <si>
+    <t>Total Shop Orders</t>
+  </si>
+  <si>
+    <t>Ramesh Agarwal</t>
+  </si>
+  <si>
+    <t>ramesh@shop.com</t>
+  </si>
+  <si>
+    <t>+91-9876543210</t>
+  </si>
+  <si>
+    <t>Ramesh General Store (BLR)</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>12, MG Road, Bengaluru</t>
   </si>
   <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>₹0.00</t>
-  </si>
-  <si>
-    <t>3/3/2026, 10:17:14 pm</t>
-  </si>
-  <si>
-    <t>3/3/2026, 10:17:53 pm</t>
-  </si>
-  <si>
-    <t>Ravi Drolia</t>
-  </si>
-  <si>
-    <t>ravio@mnit.ac.in</t>
-  </si>
-  <si>
-    <t>123123</t>
-  </si>
-  <si>
-    <t>3/3/2026, 10:20:12 pm</t>
-  </si>
-  <si>
-    <t>3/3/2026, 10:20:32 pm</t>
-  </si>
-  <si>
-    <t>Virat Kohli</t>
-  </si>
-  <si>
-    <t>virat@mnit.ac.in</t>
-  </si>
-  <si>
-    <t>110203</t>
-  </si>
-  <si>
-    <t>₹977.00</t>
-  </si>
-  <si>
-    <t>4/3/2026, 12:19:43 am</t>
-  </si>
-  <si>
-    <t>4/3/2026, 1:26:54 am</t>
-  </si>
-  <si>
-    <t>Cristiano Ronaldo</t>
-  </si>
-  <si>
-    <t>cristiano@gmail.com</t>
-  </si>
-  <si>
-    <t>4/3/2026, 7:17:02 pm</t>
-  </si>
-  <si>
-    <t>Test AutoReport</t>
-  </si>
-  <si>
-    <t>test_autoreport_520987547@example.com</t>
-  </si>
-  <si>
-    <t>4/3/2026, 7:21:46 pm</t>
-  </si>
-  <si>
-    <t>Neymar Jr</t>
-  </si>
-  <si>
-    <t>neymar@gmail.com</t>
-  </si>
-  <si>
-    <t>4/3/2026, 7:23:25 pm</t>
-  </si>
-  <si>
-    <t>Shop Name</t>
-  </si>
-  <si>
-    <t>Shop Category</t>
-  </si>
-  <si>
-    <t>Shop Address</t>
-  </si>
-  <si>
-    <t>Shop Verified</t>
-  </si>
-  <si>
-    <t>Shop Open</t>
-  </si>
-  <si>
-    <t>Shop Rating</t>
-  </si>
-  <si>
-    <t>Total Shop Orders</t>
-  </si>
-  <si>
-    <t>Ramesh Agarwal</t>
-  </si>
-  <si>
-    <t>ramesh@shop.com</t>
-  </si>
-  <si>
-    <t>+91-9876543210</t>
-  </si>
-  <si>
-    <t>Ramesh General Store</t>
-  </si>
-  <si>
-    <t>General</t>
-  </si>
-  <si>
-    <t>12, MG Road, Bengaluru</t>
+    <t>4/3/2026, 10:29:46 pm</t>
   </si>
   <si>
     <t>Priya Mehta</t>
@@ -231,31 +177,43 @@
     <t>+91-9123456789</t>
   </si>
   <si>
-    <t>Priya's Pharmacy &amp; Fresh</t>
+    <t>Priyas Pharmacy &amp; Fresh (BLR)</t>
   </si>
   <si>
     <t>45, Indiranagar, Bengaluru</t>
   </si>
   <si>
-    <t>Saarvik</t>
-  </si>
-  <si>
-    <t>saarvik@mnit.ac.in</t>
-  </si>
-  <si>
-    <t>1223456</t>
-  </si>
-  <si>
-    <t>Saarvik Athleisure</t>
-  </si>
-  <si>
-    <t>MNIT Deans Gate</t>
-  </si>
-  <si>
-    <t>3/3/2026, 5:05:44 pm</t>
-  </si>
-  <si>
-    <t>3/3/2026, 11:19:51 pm</t>
+    <t>Amit Singh</t>
+  </si>
+  <si>
+    <t>amit@shop.com</t>
+  </si>
+  <si>
+    <t>+91-9888877777</t>
+  </si>
+  <si>
+    <t>Amit SuperMart (DEL)</t>
+  </si>
+  <si>
+    <t>Connaught Place, New Delhi</t>
+  </si>
+  <si>
+    <t>Neha Joshi</t>
+  </si>
+  <si>
+    <t>neha@shop.com</t>
+  </si>
+  <si>
+    <t>+91-9111122222</t>
+  </si>
+  <si>
+    <t>Neha Organics (BOM)</t>
+  </si>
+  <si>
+    <t>Bandra West, Mumbai</t>
+  </si>
+  <si>
+    <t>4/3/2026, 10:29:47 pm</t>
   </si>
   <si>
     <t>Metric</t>
@@ -282,7 +240,7 @@
     <t>Report Generated At</t>
   </si>
   <si>
-    <t>4/3/2026, 7:23:28 pm</t>
+    <t>4/3/2026, 10:29:49 pm</t>
   </si>
 </sst>
 </file>
@@ -694,7 +652,7 @@
   <sheetPr>
     <tabColor rgb="FF4CAF50"/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -763,7 +721,7 @@
         <v>15</v>
       </c>
       <c r="G2" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>16</v>
@@ -792,25 +750,25 @@
         <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F3" t="s">
         <v>15</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="I3" t="s">
         <v>17</v>
       </c>
       <c r="J3" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K3" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -818,34 +776,34 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>14</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -853,34 +811,34 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
         <v>29</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>31</v>
       </c>
-      <c r="E5" t="s">
-        <v>14</v>
-      </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="I5" t="s">
         <v>17</v>
       </c>
       <c r="J5" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="K5" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -888,174 +846,34 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="G6" s="2">
         <v>0</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7">
-        <v>3</v>
-      </c>
-      <c r="H7" t="s">
-        <v>44</v>
-      </c>
-      <c r="I7" t="s">
-        <v>17</v>
-      </c>
-      <c r="J7" t="s">
-        <v>45</v>
-      </c>
-      <c r="K7" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="2">
-        <v>0</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9" t="s">
-        <v>33</v>
-      </c>
-      <c r="I9" t="s">
-        <v>17</v>
-      </c>
-      <c r="J9" t="s">
-        <v>52</v>
-      </c>
-      <c r="K9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G10" s="2">
-        <v>0</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>55</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1069,7 +887,7 @@
   <sheetPr>
     <tabColor rgb="FF2196F3"/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1101,25 +919,25 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>5</v>
@@ -1139,34 +957,34 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="J2" s="3">
         <v>4.6</v>
       </c>
       <c r="K2" s="3">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>15</v>
@@ -1175,10 +993,10 @@
         <v>17</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1186,34 +1004,34 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="E3" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="G3" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="H3" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="I3" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="J3">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L3" t="s">
         <v>15</v>
@@ -1222,10 +1040,10 @@
         <v>17</v>
       </c>
       <c r="N3" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="O3" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1233,46 +1051,93 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="H4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" s="3">
+        <v>3.7</v>
+      </c>
+      <c r="K4" s="3">
+        <v>0</v>
+      </c>
+      <c r="L4" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J4" s="3">
-        <v>0</v>
-      </c>
-      <c r="K4" s="3">
-        <v>1</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>32</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>17</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>80</v>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" t="s">
+        <v>65</v>
+      </c>
+      <c r="H5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J5">
+        <v>4.3</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="s">
+        <v>15</v>
+      </c>
+      <c r="M5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N5" t="s">
+        <v>66</v>
+      </c>
+      <c r="O5" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1295,50 +1160,50 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="B2">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="B3">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="B6">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1346,15 +1211,15 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="B8" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Major Bugs in Auto/Manual Location Detection in new account creation, added edit profile feature in both seller and buyer dashboard with proper rerouting of all products to new location
</commit_message>
<xml_diff>
--- a/backend/reports/users_report.xlsx
+++ b/backend/reports/users_report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="101">
   <si>
     <t>#</t>
   </si>
@@ -63,27 +63,33 @@
     <t>No</t>
   </si>
   <si>
+    <t>₹723.00</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>4/3/2026, 10:29:44 pm</t>
+  </si>
+  <si>
+    <t>4/3/2026, 10:37:03 pm</t>
+  </si>
+  <si>
+    <t>Sneha Rao</t>
+  </si>
+  <si>
+    <t>sneha@buyer.com</t>
+  </si>
+  <si>
+    <t>+91-9988776666</t>
+  </si>
+  <si>
+    <t>Domlur, Bengaluru</t>
+  </si>
+  <si>
     <t>₹0.00</t>
   </si>
   <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>4/3/2026, 10:29:44 pm</t>
-  </si>
-  <si>
-    <t>Sneha Rao</t>
-  </si>
-  <si>
-    <t>sneha@buyer.com</t>
-  </si>
-  <si>
-    <t>+91-9988776666</t>
-  </si>
-  <si>
-    <t>Domlur, Bengaluru</t>
-  </si>
-  <si>
     <t>Rohan Gupta</t>
   </si>
   <si>
@@ -111,6 +117,15 @@
     <t>Colaba, Mumbai</t>
   </si>
   <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>₹191.00</t>
+  </si>
+  <si>
+    <t>6/3/2026, 8:27:47 pm</t>
+  </si>
+  <si>
     <t>Jaipur User</t>
   </si>
   <si>
@@ -123,6 +138,27 @@
     <t>C-Scheme, Jaipur, Rajasthan</t>
   </si>
   <si>
+    <t>4/3/2026, 10:37:04 pm</t>
+  </si>
+  <si>
+    <t>New User Jaipur 1 (changed to Mumbai)</t>
+  </si>
+  <si>
+    <t>jaipur1@buyer.com</t>
+  </si>
+  <si>
+    <t>6391929191</t>
+  </si>
+  <si>
+    <t>Film City</t>
+  </si>
+  <si>
+    <t>8/3/2026, 1:55:40 am</t>
+  </si>
+  <si>
+    <t>8/3/2026, 3:06:54 am</t>
+  </si>
+  <si>
     <t>Shop Name</t>
   </si>
   <si>
@@ -162,9 +198,6 @@
     <t>12, MG Road, Bengaluru</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>4/3/2026, 10:29:46 pm</t>
   </si>
   <si>
@@ -183,6 +216,9 @@
     <t>45, Indiranagar, Bengaluru</t>
   </si>
   <si>
+    <t>4/3/2026, 10:37:05 pm</t>
+  </si>
+  <si>
     <t>Amit Singh</t>
   </si>
   <si>
@@ -216,6 +252,45 @@
     <t>4/3/2026, 10:29:47 pm</t>
   </si>
   <si>
+    <t>Jaipur Seller 1</t>
+  </si>
+  <si>
+    <t>jaipur1@shop.com</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>Jaipur Sports Shop 1</t>
+  </si>
+  <si>
+    <t>MNIT Deans Gate</t>
+  </si>
+  <si>
+    <t>8/3/2026, 2:02:41 am</t>
+  </si>
+  <si>
+    <t>8/3/2026, 2:06:21 am</t>
+  </si>
+  <si>
+    <t>Jaipur Seller 2</t>
+  </si>
+  <si>
+    <t>jaipur2@shop.com</t>
+  </si>
+  <si>
+    <t>1010101010</t>
+  </si>
+  <si>
+    <t>Jaipur Store Test 2</t>
+  </si>
+  <si>
+    <t>8/3/2026, 2:27:33 am</t>
+  </si>
+  <si>
+    <t>8/3/2026, 2:27:49 am</t>
+  </si>
+  <si>
     <t>Metric</t>
   </si>
   <si>
@@ -240,7 +315,7 @@
     <t>Report Generated At</t>
   </si>
   <si>
-    <t>4/3/2026, 10:29:49 pm</t>
+    <t>8/3/2026, 3:06:56 am</t>
   </si>
 </sst>
 </file>
@@ -652,7 +727,7 @@
   <sheetPr>
     <tabColor rgb="FF4CAF50"/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -721,7 +796,7 @@
         <v>15</v>
       </c>
       <c r="G2" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>16</v>
@@ -733,7 +808,7 @@
         <v>18</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -741,16 +816,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F3" t="s">
         <v>15</v>
@@ -759,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I3" t="s">
         <v>17</v>
@@ -768,7 +843,7 @@
         <v>18</v>
       </c>
       <c r="K3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -776,16 +851,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>15</v>
@@ -794,16 +869,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -811,34 +886,34 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="I5" t="s">
         <v>17</v>
       </c>
       <c r="J5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K5" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -846,16 +921,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>15</v>
@@ -864,16 +939,51 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>27</v>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" t="s">
+        <v>46</v>
+      </c>
+      <c r="K7" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -887,7 +997,7 @@
   <sheetPr>
     <tabColor rgb="FF2196F3"/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -919,25 +1029,25 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>5</v>
@@ -957,34 +1067,34 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="J2" s="3">
         <v>4.6</v>
       </c>
       <c r="K2" s="3">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>15</v>
@@ -993,10 +1103,10 @@
         <v>17</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1004,34 +1114,34 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="D3" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="F3" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="H3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="J3">
         <v>4.5</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L3" t="s">
         <v>15</v>
@@ -1040,10 +1150,10 @@
         <v>17</v>
       </c>
       <c r="N3" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="O3" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1051,28 +1161,28 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>47</v>
-      </c>
       <c r="G4" s="3" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="J4" s="3">
         <v>3.7</v>
@@ -1087,10 +1197,10 @@
         <v>17</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1098,34 +1208,34 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="E5" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="F5" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="G5" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="H5" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I5" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="J5">
         <v>4.3</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L5" t="s">
         <v>15</v>
@@ -1134,10 +1244,104 @@
         <v>17</v>
       </c>
       <c r="N5" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="O5" t="s">
-        <v>66</v>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="3">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3">
+        <v>0</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="O6" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" t="s">
+        <v>83</v>
+      </c>
+      <c r="H7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7" t="s">
+        <v>34</v>
+      </c>
+      <c r="M7" t="s">
+        <v>17</v>
+      </c>
+      <c r="N7" t="s">
+        <v>90</v>
+      </c>
+      <c r="O7" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1160,50 +1364,50 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="B2">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1211,15 +1415,15 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Distance Calculation logic
</commit_message>
<xml_diff>
--- a/backend/reports/users_report.xlsx
+++ b/backend/reports/users_report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="116">
   <si>
     <t>#</t>
   </si>
@@ -30,6 +30,9 @@
     <t>Address</t>
   </si>
   <si>
+    <t>PIN Code</t>
+  </si>
+  <si>
     <t>Face ID Enrolled</t>
   </si>
   <si>
@@ -57,39 +60,51 @@
     <t>+91-9988776655</t>
   </si>
   <si>
-    <t>Brigade Road, Bengaluru</t>
+    <t>Indira Road</t>
+  </si>
+  <si>
+    <t>110001</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>₹1727.00</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>4/3/2026, 10:29:44 pm</t>
+  </si>
+  <si>
+    <t>8/3/2026, 12:48:37 pm</t>
+  </si>
+  <si>
+    <t>Sneha Rao</t>
+  </si>
+  <si>
+    <t>sneha@buyer.com</t>
+  </si>
+  <si>
+    <t>+91-9988776666</t>
+  </si>
+  <si>
+    <t>Domlur, Bengaluru</t>
+  </si>
+  <si>
+    <t>—</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>₹723.00</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>4/3/2026, 10:29:44 pm</t>
+    <t>₹0.00</t>
   </si>
   <si>
     <t>4/3/2026, 10:37:03 pm</t>
   </si>
   <si>
-    <t>Sneha Rao</t>
-  </si>
-  <si>
-    <t>sneha@buyer.com</t>
-  </si>
-  <si>
-    <t>+91-9988776666</t>
-  </si>
-  <si>
-    <t>Domlur, Bengaluru</t>
-  </si>
-  <si>
-    <t>₹0.00</t>
-  </si>
-  <si>
     <t>Rohan Gupta</t>
   </si>
   <si>
@@ -102,6 +117,9 @@
     <t>India Gate vicinity, New Delhi</t>
   </si>
   <si>
+    <t>₹255.00</t>
+  </si>
+  <si>
     <t>4/3/2026, 10:29:45 pm</t>
   </si>
   <si>
@@ -117,9 +135,6 @@
     <t>Colaba, Mumbai</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>₹191.00</t>
   </si>
   <si>
@@ -138,6 +153,9 @@
     <t>C-Scheme, Jaipur, Rajasthan</t>
   </si>
   <si>
+    <t>302001</t>
+  </si>
+  <si>
     <t>4/3/2026, 10:37:04 pm</t>
   </si>
   <si>
@@ -153,12 +171,30 @@
     <t>Film City</t>
   </si>
   <si>
+    <t>400050</t>
+  </si>
+  <si>
     <t>8/3/2026, 1:55:40 am</t>
   </si>
   <si>
     <t>8/3/2026, 3:06:54 am</t>
   </si>
   <si>
+    <t>Vaibhav</t>
+  </si>
+  <si>
+    <t>vaibhav@buyer.com</t>
+  </si>
+  <si>
+    <t>191919191919</t>
+  </si>
+  <si>
+    <t>Jaipur Municipal Corporation, Sanganer Tehsil, Jaipur, Rajasthan, 302014, India</t>
+  </si>
+  <si>
+    <t>8/3/2026, 12:56:16 pm</t>
+  </si>
+  <si>
     <t>Shop Name</t>
   </si>
   <si>
@@ -168,6 +204,9 @@
     <t>Shop Address</t>
   </si>
   <si>
+    <t>Shop PIN Code</t>
+  </si>
+  <si>
     <t>Shop Verified</t>
   </si>
   <si>
@@ -198,6 +237,9 @@
     <t>12, MG Road, Bengaluru</t>
   </si>
   <si>
+    <t>560001</t>
+  </si>
+  <si>
     <t>4/3/2026, 10:29:46 pm</t>
   </si>
   <si>
@@ -216,6 +258,9 @@
     <t>45, Indiranagar, Bengaluru</t>
   </si>
   <si>
+    <t>560038</t>
+  </si>
+  <si>
     <t>4/3/2026, 10:37:05 pm</t>
   </si>
   <si>
@@ -282,7 +327,7 @@
     <t>1010101010</t>
   </si>
   <si>
-    <t>Jaipur Store Test 2</t>
+    <t>Jaipur Store Test 2 (changed to Delhi)</t>
   </si>
   <si>
     <t>8/3/2026, 2:27:33 am</t>
@@ -315,7 +360,7 @@
     <t>Report Generated At</t>
   </si>
   <si>
-    <t>8/3/2026, 3:06:56 am</t>
+    <t>8/3/2026, 12:56:18 pm</t>
   </si>
 </sst>
 </file>
@@ -727,7 +772,7 @@
   <sheetPr>
     <tabColor rgb="FF4CAF50"/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -735,13 +780,14 @@
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="35" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="9" width="16" customWidth="1"/>
-    <col min="10" max="11" width="22" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="10" width="16" customWidth="1"/>
+    <col min="11" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -775,215 +821,274 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="2">
-        <v>4</v>
-      </c>
-      <c r="H2" s="2" t="s">
         <v>16</v>
       </c>
+      <c r="G2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="2">
+        <v>5</v>
+      </c>
       <c r="I2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" t="s">
         <v>20</v>
       </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="2">
-        <v>0</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>24</v>
+      <c r="H4" s="2">
+        <v>1</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="J4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5">
+        <v>26</v>
+      </c>
+      <c r="G5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5">
         <v>1</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5" t="s">
         <v>35</v>
       </c>
-      <c r="I5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" t="s">
-        <v>29</v>
-      </c>
-      <c r="K5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="2">
+        <v>46</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="2">
         <v>0</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="I6" s="2" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
-      </c>
-      <c r="G7">
+        <v>52</v>
+      </c>
+      <c r="G7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7">
         <v>0</v>
       </c>
-      <c r="H7" t="s">
-        <v>24</v>
-      </c>
       <c r="I7" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="J7" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="K7" t="s">
-        <v>47</v>
+        <v>53</v>
+      </c>
+      <c r="L7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -997,7 +1102,7 @@
   <sheetPr>
     <tabColor rgb="FF2196F3"/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1007,15 +1112,16 @@
     <col min="5" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="35" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="12" width="18" customWidth="1"/>
-    <col min="13" max="13" width="16" customWidth="1"/>
-    <col min="14" max="15" width="22" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="12" max="13" width="18" customWidth="1"/>
+    <col min="14" max="14" width="16" customWidth="1"/>
+    <col min="15" max="16" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1029,31 +1135,31 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>5</v>
+        <v>67</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>9</v>
@@ -1061,287 +1167,308 @@
       <c r="O1" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" s="3">
+        <v>17</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" s="3">
         <v>4.6</v>
       </c>
-      <c r="K2" s="3">
-        <v>6</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>15</v>
+      <c r="L2" s="3">
+        <v>9</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="F3" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G3" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="H3" t="s">
-        <v>34</v>
+        <v>81</v>
       </c>
       <c r="I3" t="s">
-        <v>34</v>
-      </c>
-      <c r="J3">
+        <v>17</v>
+      </c>
+      <c r="J3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3">
         <v>4.5</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>4</v>
       </c>
-      <c r="L3" t="s">
-        <v>15</v>
-      </c>
       <c r="M3" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="N3" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="O3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="P3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="J4" s="3">
+        <v>17</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="3">
         <v>3.7</v>
       </c>
-      <c r="K4" s="3">
-        <v>0</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>15</v>
+      <c r="L4" s="3">
+        <v>3</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C5" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="D5" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="E5" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G5" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="I5" t="s">
-        <v>34</v>
-      </c>
-      <c r="J5">
+        <v>17</v>
+      </c>
+      <c r="J5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K5">
         <v>4.3</v>
       </c>
-      <c r="K5">
-        <v>3</v>
-      </c>
-      <c r="L5" t="s">
-        <v>15</v>
+      <c r="L5">
+        <v>6</v>
       </c>
       <c r="M5" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="N5" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="O5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+      <c r="P5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="J6" s="3">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="K6" s="3">
         <v>0</v>
       </c>
-      <c r="L6" s="3" t="s">
-        <v>15</v>
+      <c r="L6" s="3">
+        <v>0</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>84</v>
+        <v>19</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="E7" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="F7" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G7" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="H7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I7" t="s">
-        <v>34</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="J7" t="s">
+        <v>17</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
-      <c r="L7" t="s">
-        <v>34</v>
+      <c r="L7">
+        <v>0</v>
       </c>
       <c r="M7" t="s">
         <v>17</v>
       </c>
       <c r="N7" t="s">
-        <v>90</v>
+        <v>19</v>
       </c>
       <c r="O7" t="s">
-        <v>91</v>
+        <v>105</v>
+      </c>
+      <c r="P7" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -1364,31 +1491,31 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="B2">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -1396,15 +1523,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="B6">
         <v>6</v>
@@ -1412,18 +1539,18 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Implemented smart cart splitting, delivery optimization, and advanced cart UI
</commit_message>
<xml_diff>
--- a/backend/reports/users_report.xlsx
+++ b/backend/reports/users_report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="117">
   <si>
     <t>#</t>
   </si>
@@ -69,7 +69,7 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>₹1727.00</t>
+    <t>₹3970.00</t>
   </si>
   <si>
     <t>Active</t>
@@ -195,6 +195,9 @@
     <t>8/3/2026, 12:56:16 pm</t>
   </si>
   <si>
+    <t>8/3/2026, 12:56:22 pm</t>
+  </si>
+  <si>
     <t>Shop Name</t>
   </si>
   <si>
@@ -360,7 +363,7 @@
     <t>Report Generated At</t>
   </si>
   <si>
-    <t>8/3/2026, 12:56:18 pm</t>
+    <t>9/3/2026, 4:17:50 pm</t>
   </si>
 </sst>
 </file>
@@ -848,7 +851,7 @@
         <v>17</v>
       </c>
       <c r="H2" s="2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>18</v>
@@ -1073,7 +1076,7 @@
         <v>26</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="H8" s="2">
         <v>0</v>
@@ -1088,7 +1091,7 @@
         <v>59</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1135,28 +1138,28 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>6</v>
@@ -1176,25 +1179,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>17</v>
@@ -1215,7 +1218,7 @@
         <v>19</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>47</v>
@@ -1226,25 +1229,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I3" t="s">
         <v>17</v>
@@ -1265,10 +1268,10 @@
         <v>19</v>
       </c>
       <c r="O3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -1276,22 +1279,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>16</v>
@@ -1306,7 +1309,7 @@
         <v>3.7</v>
       </c>
       <c r="L4" s="3">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>27</v>
@@ -1315,10 +1318,10 @@
         <v>19</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -1326,22 +1329,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H5" t="s">
         <v>52</v>
@@ -1365,10 +1368,10 @@
         <v>19</v>
       </c>
       <c r="O5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="P5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -1376,22 +1379,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>26</v>
@@ -1415,10 +1418,10 @@
         <v>19</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -1426,19 +1429,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G7" t="s">
         <v>15</v>
@@ -1456,7 +1459,7 @@
         <v>0</v>
       </c>
       <c r="L7">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M7" t="s">
         <v>17</v>
@@ -1465,10 +1468,10 @@
         <v>19</v>
       </c>
       <c r="O7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="P7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1491,15 +1494,15 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B2">
         <v>13</v>
@@ -1507,7 +1510,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B3">
         <v>7</v>
@@ -1515,7 +1518,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -1523,15 +1526,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B6">
         <v>6</v>
@@ -1542,15 +1545,15 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implemented accurate map-based location selection using Leaflet and OpenStreetMap with 3-step registration flow and saved addresses
</commit_message>
<xml_diff>
--- a/backend/reports/users_report.xlsx
+++ b/backend/reports/users_report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="120">
   <si>
     <t>#</t>
   </si>
@@ -198,6 +198,18 @@
     <t>8/3/2026, 12:56:22 pm</t>
   </si>
   <si>
+    <t>Jaipur Account for Map Integration</t>
+  </si>
+  <si>
+    <t>jaipur_v1@buyer.com</t>
+  </si>
+  <si>
+    <t>1010101010</t>
+  </si>
+  <si>
+    <t>9/3/2026, 4:54:27 pm</t>
+  </si>
+  <si>
     <t>Shop Name</t>
   </si>
   <si>
@@ -327,9 +339,6 @@
     <t>jaipur2@shop.com</t>
   </si>
   <si>
-    <t>1010101010</t>
-  </si>
-  <si>
     <t>Jaipur Store Test 2 (changed to Delhi)</t>
   </si>
   <si>
@@ -363,7 +372,7 @@
     <t>Report Generated At</t>
   </si>
   <si>
-    <t>9/3/2026, 4:17:50 pm</t>
+    <t>9/3/2026, 4:54:32 pm</t>
   </si>
 </sst>
 </file>
@@ -775,7 +784,7 @@
   <sheetPr>
     <tabColor rgb="FF4CAF50"/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1092,6 +1101,44 @@
       </c>
       <c r="L8" s="2" t="s">
         <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9" t="s">
+        <v>64</v>
+      </c>
+      <c r="L9" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1138,28 +1185,28 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>6</v>
@@ -1179,25 +1226,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>17</v>
@@ -1218,7 +1265,7 @@
         <v>19</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>47</v>
@@ -1229,25 +1276,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" t="s">
         <v>77</v>
       </c>
-      <c r="C3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" t="s">
-        <v>79</v>
-      </c>
-      <c r="E3" t="s">
-        <v>80</v>
-      </c>
-      <c r="F3" t="s">
-        <v>73</v>
-      </c>
       <c r="G3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="H3" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="I3" t="s">
         <v>17</v>
@@ -1268,10 +1315,10 @@
         <v>19</v>
       </c>
       <c r="O3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="P3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -1279,22 +1326,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>16</v>
@@ -1318,10 +1365,10 @@
         <v>19</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -1329,22 +1376,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="H5" t="s">
         <v>52</v>
@@ -1368,10 +1415,10 @@
         <v>19</v>
       </c>
       <c r="O5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="P5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -1379,22 +1426,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>26</v>
@@ -1418,10 +1465,10 @@
         <v>19</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -1429,19 +1476,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D7" t="s">
-        <v>104</v>
+        <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="F7" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G7" t="s">
         <v>15</v>
@@ -1468,10 +1515,10 @@
         <v>19</v>
       </c>
       <c r="O7" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="P7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -1494,31 +1541,31 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B2">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -1526,7 +1573,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B5">
         <v>5</v>
@@ -1534,7 +1581,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B6">
         <v>6</v>
@@ -1550,10 +1597,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B8" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improved Shop/Category Filters, supporting multi-select with local first option
</commit_message>
<xml_diff>
--- a/backend/reports/users_report.xlsx
+++ b/backend/reports/users_report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="123">
   <si>
     <t>#</t>
   </si>
@@ -60,7 +60,7 @@
     <t>+91-9988776655</t>
   </si>
   <si>
-    <t>Indira Road</t>
+    <t>Indira Road, Central Delhi, Delhi - 110001</t>
   </si>
   <si>
     <t>110001</t>
@@ -90,7 +90,7 @@
     <t>+91-9988776666</t>
   </si>
   <si>
-    <t>Domlur, Bengaluru</t>
+    <t xml:space="preserve">Domlur, Bengaluru,  - </t>
   </si>
   <si>
     <t>—</t>
@@ -114,7 +114,7 @@
     <t>+91-9988776677</t>
   </si>
   <si>
-    <t>India Gate vicinity, New Delhi</t>
+    <t xml:space="preserve">India Gate vicinity, New Delhi,  - </t>
   </si>
   <si>
     <t>₹255.00</t>
@@ -132,7 +132,7 @@
     <t>+91-9988776688</t>
   </si>
   <si>
-    <t>Colaba, Mumbai</t>
+    <t xml:space="preserve">Colaba, Mumbai,  - </t>
   </si>
   <si>
     <t>₹191.00</t>
@@ -150,7 +150,7 @@
     <t>+91-9000000000</t>
   </si>
   <si>
-    <t>C-Scheme, Jaipur, Rajasthan</t>
+    <t>C-Scheme, Jaipur, Rajasthan, Jaipur, Rajasthan - 302001</t>
   </si>
   <si>
     <t>302001</t>
@@ -168,7 +168,7 @@
     <t>6391929191</t>
   </si>
   <si>
-    <t>Film City</t>
+    <t>Film City, Mumbai, Maharashtra - 400050</t>
   </si>
   <si>
     <t>400050</t>
@@ -189,7 +189,7 @@
     <t>191919191919</t>
   </si>
   <si>
-    <t>Jaipur Municipal Corporation, Sanganer Tehsil, Jaipur, Rajasthan, 302014, India</t>
+    <t xml:space="preserve">Jaipur Municipal Corporation, Sanganer Tehsil, Jaipur, Rajasthan, 302014, India,  - </t>
   </si>
   <si>
     <t>8/3/2026, 12:56:16 pm</t>
@@ -207,9 +207,15 @@
     <t>1010101010</t>
   </si>
   <si>
+    <t>₹1059.00</t>
+  </si>
+  <si>
     <t>9/3/2026, 4:54:27 pm</t>
   </si>
   <si>
+    <t>9/3/2026, 4:54:35 pm</t>
+  </si>
+  <si>
     <t>Shop Name</t>
   </si>
   <si>
@@ -249,7 +255,7 @@
     <t>General</t>
   </si>
   <si>
-    <t>12, MG Road, Bengaluru</t>
+    <t>12, MG Road, Bengaluru, Bengaluru,  - 560001</t>
   </si>
   <si>
     <t>560001</t>
@@ -270,7 +276,7 @@
     <t>Priyas Pharmacy &amp; Fresh (BLR)</t>
   </si>
   <si>
-    <t>45, Indiranagar, Bengaluru</t>
+    <t>45, Indiranagar, Bengaluru, Bengaluru,  - 560038</t>
   </si>
   <si>
     <t>560038</t>
@@ -291,7 +297,7 @@
     <t>Amit SuperMart (DEL)</t>
   </si>
   <si>
-    <t>Connaught Place, New Delhi</t>
+    <t>Connaught Place, New Delhi, New Delhi,  - 110001</t>
   </si>
   <si>
     <t>Neha Joshi</t>
@@ -306,7 +312,7 @@
     <t>Neha Organics (BOM)</t>
   </si>
   <si>
-    <t>Bandra West, Mumbai</t>
+    <t>Bandra West, Mumbai, Mumbai,  - 400050</t>
   </si>
   <si>
     <t>4/3/2026, 10:29:47 pm</t>
@@ -324,7 +330,10 @@
     <t>Jaipur Sports Shop 1</t>
   </si>
   <si>
-    <t>MNIT Deans Gate</t>
+    <t>MNIT Deans Gate, Jaipur Municipal Corporation, Rajasthan - 302018</t>
+  </si>
+  <si>
+    <t>302018</t>
   </si>
   <si>
     <t>8/3/2026, 2:02:41 am</t>
@@ -372,7 +381,7 @@
     <t>Report Generated At</t>
   </si>
   <si>
-    <t>9/3/2026, 4:54:32 pm</t>
+    <t>9/3/2026, 5:49:17 pm</t>
   </si>
 </sst>
 </file>
@@ -1123,22 +1132,22 @@
         <v>26</v>
       </c>
       <c r="G9" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="s">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="J9" t="s">
         <v>19</v>
       </c>
       <c r="K9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1185,28 +1194,28 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>6</v>
@@ -1226,25 +1235,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>17</v>
@@ -1265,7 +1274,7 @@
         <v>19</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>47</v>
@@ -1276,25 +1285,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I3" t="s">
         <v>17</v>
@@ -1315,10 +1324,10 @@
         <v>19</v>
       </c>
       <c r="O3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="P3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -1326,22 +1335,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>16</v>
@@ -1356,7 +1365,7 @@
         <v>3.7</v>
       </c>
       <c r="L4" s="3">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>27</v>
@@ -1365,10 +1374,10 @@
         <v>19</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -1376,22 +1385,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H5" t="s">
         <v>52</v>
@@ -1415,10 +1424,10 @@
         <v>19</v>
       </c>
       <c r="O5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="P5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -1426,25 +1435,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>26</v>
+        <v>106</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>27</v>
@@ -1465,10 +1474,10 @@
         <v>19</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -1476,19 +1485,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D7" t="s">
         <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G7" t="s">
         <v>15</v>
@@ -1515,10 +1524,10 @@
         <v>19</v>
       </c>
       <c r="O7" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="P7" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1541,15 +1550,15 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B2">
         <v>14</v>
@@ -1557,7 +1566,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B3">
         <v>8</v>
@@ -1565,7 +1574,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -1573,15 +1582,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B6">
         <v>6</v>
@@ -1592,15 +1601,15 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Initial commit to add project structure
</commit_message>
<xml_diff>
--- a/backend/reports/users_report.xlsx
+++ b/backend/reports/users_report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="128">
   <si>
     <t>#</t>
   </si>
@@ -216,6 +216,21 @@
     <t>9/3/2026, 4:54:35 pm</t>
   </si>
   <si>
+    <t>Ravi</t>
+  </si>
+  <si>
+    <t>ravi@buyer.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calgiri Road, Jaipur Municipal Corporation, Sanganer Tehsil, Jaipur, Rajasthan, 302014, India,  - </t>
+  </si>
+  <si>
+    <t>₹1195.00</t>
+  </si>
+  <si>
+    <t>9/3/2026, 6:39:54 pm</t>
+  </si>
+  <si>
     <t>Shop Name</t>
   </si>
   <si>
@@ -381,7 +396,7 @@
     <t>Report Generated At</t>
   </si>
   <si>
-    <t>9/3/2026, 5:49:17 pm</t>
+    <t>9/3/2026, 6:43:54 pm</t>
   </si>
 </sst>
 </file>
@@ -793,7 +808,7 @@
   <sheetPr>
     <tabColor rgb="FF4CAF50"/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1148,6 +1163,44 @@
       </c>
       <c r="L9" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="2">
+        <v>1</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1194,28 +1247,28 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>6</v>
@@ -1235,25 +1288,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>17</v>
@@ -1265,7 +1318,7 @@
         <v>4.6</v>
       </c>
       <c r="L2" s="3">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>27</v>
@@ -1274,7 +1327,7 @@
         <v>19</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>47</v>
@@ -1285,25 +1338,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E3" t="s">
+        <v>91</v>
+      </c>
+      <c r="F3" t="s">
         <v>84</v>
       </c>
-      <c r="D3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F3" t="s">
-        <v>79</v>
-      </c>
       <c r="G3" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="H3" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="I3" t="s">
         <v>17</v>
@@ -1315,7 +1368,7 @@
         <v>4.5</v>
       </c>
       <c r="L3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M3" t="s">
         <v>27</v>
@@ -1324,10 +1377,10 @@
         <v>19</v>
       </c>
       <c r="O3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="P3" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -1335,22 +1388,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>16</v>
@@ -1365,7 +1418,7 @@
         <v>3.7</v>
       </c>
       <c r="L4" s="3">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>27</v>
@@ -1374,10 +1427,10 @@
         <v>19</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -1385,22 +1438,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D5" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="E5" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="F5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="G5" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="H5" t="s">
         <v>52</v>
@@ -1415,7 +1468,7 @@
         <v>4.3</v>
       </c>
       <c r="L5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M5" t="s">
         <v>27</v>
@@ -1424,10 +1477,10 @@
         <v>19</v>
       </c>
       <c r="O5" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="P5" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -1435,25 +1488,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>27</v>
@@ -1474,10 +1527,10 @@
         <v>19</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -1485,19 +1538,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C7" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D7" t="s">
         <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="F7" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="G7" t="s">
         <v>15</v>
@@ -1515,7 +1568,7 @@
         <v>0</v>
       </c>
       <c r="L7">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M7" t="s">
         <v>17</v>
@@ -1524,10 +1577,10 @@
         <v>19</v>
       </c>
       <c r="O7" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="P7" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -1550,31 +1603,31 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B2">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B3">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -1582,7 +1635,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B5">
         <v>6</v>
@@ -1590,7 +1643,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B6">
         <v>6</v>
@@ -1601,15 +1654,15 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B8" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ui): improve dashboard layouts, fix cart & carousel scrolling, enhance shop headers and seller UI
- Fixed cart internal scroll behavior (prevent page scroll chaining)
- Implemented horizontal scrolling for product carousels
- Centered main content across dashboards and forms
- Improved seller dashboard layout and added contextual widgets
- Redesigned shop headers with richer metadata (rating, distance, ETA)
- Added ambient background animations and UI polish
</commit_message>
<xml_diff>
--- a/backend/reports/users_report.xlsx
+++ b/backend/reports/users_report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="136">
   <si>
     <t>#</t>
   </si>
@@ -69,7 +69,7 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>₹3970.00</t>
+    <t>₹7049.00</t>
   </si>
   <si>
     <t>Active</t>
@@ -231,6 +231,30 @@
     <t>9/3/2026, 6:39:54 pm</t>
   </si>
   <si>
+    <t>Ravi 2</t>
+  </si>
+  <si>
+    <t>ravi2@buyer.com</t>
+  </si>
+  <si>
+    <t>10101010101</t>
+  </si>
+  <si>
+    <t>9/3/2026, 9:48:22 pm</t>
+  </si>
+  <si>
+    <t>9/3/2026, 9:49:14 pm</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>a@buyer.com</t>
+  </si>
+  <si>
+    <t>9/3/2026, 10:51:18 pm</t>
+  </si>
+  <si>
     <t>Shop Name</t>
   </si>
   <si>
@@ -396,7 +420,7 @@
     <t>Report Generated At</t>
   </si>
   <si>
-    <t>9/3/2026, 6:43:54 pm</t>
+    <t>9/3/2026, 11:15:41 pm</t>
   </si>
 </sst>
 </file>
@@ -808,7 +832,7 @@
   <sheetPr>
     <tabColor rgb="FF4CAF50"/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -884,7 +908,7 @@
         <v>17</v>
       </c>
       <c r="H2" s="2">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>18</v>
@@ -1201,6 +1225,82 @@
       </c>
       <c r="L10" s="2" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11" t="s">
+        <v>28</v>
+      </c>
+      <c r="J11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K11" t="s">
+        <v>75</v>
+      </c>
+      <c r="L11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1247,28 +1347,28 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>6</v>
@@ -1288,25 +1388,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>17</v>
@@ -1318,7 +1418,7 @@
         <v>4.6</v>
       </c>
       <c r="L2" s="3">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>27</v>
@@ -1327,7 +1427,7 @@
         <v>19</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>47</v>
@@ -1338,25 +1438,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="E3" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="F3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G3" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="H3" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="I3" t="s">
         <v>17</v>
@@ -1368,7 +1468,7 @@
         <v>4.5</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M3" t="s">
         <v>27</v>
@@ -1377,10 +1477,10 @@
         <v>19</v>
       </c>
       <c r="O3" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="P3" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -1388,22 +1488,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>16</v>
@@ -1418,7 +1518,7 @@
         <v>3.7</v>
       </c>
       <c r="L4" s="3">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>27</v>
@@ -1427,10 +1527,10 @@
         <v>19</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -1438,22 +1538,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="D5" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="E5" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="F5" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G5" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="H5" t="s">
         <v>52</v>
@@ -1468,7 +1568,7 @@
         <v>4.3</v>
       </c>
       <c r="L5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M5" t="s">
         <v>27</v>
@@ -1477,10 +1577,10 @@
         <v>19</v>
       </c>
       <c r="O5" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="P5" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -1488,25 +1588,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>27</v>
@@ -1518,7 +1618,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>27</v>
@@ -1527,10 +1627,10 @@
         <v>19</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -1538,19 +1638,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C7" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="D7" t="s">
         <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="F7" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G7" t="s">
         <v>15</v>
@@ -1568,7 +1668,7 @@
         <v>0</v>
       </c>
       <c r="L7">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="M7" t="s">
         <v>17</v>
@@ -1577,10 +1677,10 @@
         <v>19</v>
       </c>
       <c r="O7" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="P7" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1603,31 +1703,31 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B2">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="B3">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -1635,15 +1735,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B5">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B6">
         <v>6</v>
@@ -1654,15 +1754,15 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="B8" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
First Commit after Merging All Branches (for Project Phase A Demo)
</commit_message>
<xml_diff>
--- a/backend/reports/users_report.xlsx
+++ b/backend/reports/users_report.xlsx
@@ -69,7 +69,7 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>₹12295.00</t>
+    <t>₹14331.00</t>
   </si>
   <si>
     <t>Active</t>
@@ -78,7 +78,7 @@
     <t>4/3/2026, 10:29:44 pm</t>
   </si>
   <si>
-    <t>10/3/2026, 9:10:15 pm</t>
+    <t>13/3/2026, 1:13:28 pm</t>
   </si>
   <si>
     <t>Sneha Rao</t>
@@ -456,7 +456,7 @@
     <t>Report Generated At</t>
   </si>
   <si>
-    <t>13/3/2026, 1:11:45 pm</t>
+    <t>13/3/2026, 1:45:00 pm</t>
   </si>
 </sst>
 </file>
@@ -944,7 +944,7 @@
         <v>17</v>
       </c>
       <c r="H2" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>18</v>
@@ -1630,7 +1630,7 @@
         <v>3.7</v>
       </c>
       <c r="L4" s="3">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>27</v>
@@ -1680,7 +1680,7 @@
         <v>4.3</v>
       </c>
       <c r="L5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M5" t="s">
         <v>27</v>
@@ -1730,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="3">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>27</v>
@@ -1780,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="L7">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M7" t="s">
         <v>17</v>
@@ -1866,7 +1866,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>